<commit_message>
feat: update assessment terminology from 'Failed' to 'Needs practice' across documentation and codebase
</commit_message>
<xml_diff>
--- a/bakeit-instructor-dashboard/public/assets/reports/section-report-example.xlsx
+++ b/bakeit-instructor-dashboard/public/assets/reports/section-report-example.xlsx
@@ -378,7 +378,7 @@
       </c>
       <c r="L7" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Failed</t>
+          <t xml:space="preserve">Needs practice</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Failed</t>
+          <t xml:space="preserve">Needs practice</t>
         </is>
       </c>
     </row>

</xml_diff>